<commit_message>
Implement patches 10 through 12
</commit_message>
<xml_diff>
--- a/docs/design/weapons-passives-balance.xlsx
+++ b/docs/design/weapons-passives-balance.xlsx
@@ -649,301 +649,301 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="10" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="42" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="80" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Primary Weapons — Base Stats</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="36" t="str">
-        <x:v>Weapon</x:v>
-      </x:c>
-      <x:c r="B3" s="36" t="str">
-        <x:v>Behavior</x:v>
-      </x:c>
-      <x:c r="C3" s="36" t="str">
-        <x:v>Tags</x:v>
-      </x:c>
-      <x:c r="D3" s="36" t="str">
-        <x:v>Base Dmg</x:v>
-      </x:c>
-      <x:c r="E3" s="36" t="str">
-        <x:v>Base FR</x:v>
-      </x:c>
-      <x:c r="F3" s="36" t="str">
-        <x:v>Projectile Spd</x:v>
-      </x:c>
-      <x:c r="G3" s="36" t="str">
-        <x:v>Range</x:v>
-      </x:c>
-      <x:c r="H3" s="36" t="str">
-        <x:v>Area</x:v>
-      </x:c>
-      <x:c r="I3" s="36" t="str">
-        <x:v>Amount</x:v>
-      </x:c>
-      <x:c r="J3" s="36" t="str">
-        <x:v>Spread</x:v>
-      </x:c>
-      <x:c r="K3" s="36" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-      <x:c r="L3" s="36" t="str">
-        <x:v>Source URL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="37" t="str">
-        <x:v>Rifle</x:v>
-      </x:c>
-      <x:c r="B4" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="C4" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="D4" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E4" s="40" t="n">
-        <x:v>4.62962962962963</x:v>
-      </x:c>
-      <x:c r="F4" s="40" t="n">
-        <x:v>540</x:v>
-      </x:c>
-      <x:c r="G4" s="40" t="n">
-        <x:v>520</x:v>
-      </x:c>
-      <x:c r="H4" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="I4" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J4" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K4" s="37" t="str"/>
-      <x:c r="L4" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="37" t="str">
-        <x:v>Scatter</x:v>
-      </x:c>
-      <x:c r="B5" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="C5" s="37" t="str">
-        <x:v>projectile, spread</x:v>
-      </x:c>
-      <x:c r="D5" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E5" s="40" t="n">
-        <x:v>3.42935528120713</x:v>
-      </x:c>
-      <x:c r="F5" s="40" t="n">
-        <x:v>513</x:v>
-      </x:c>
-      <x:c r="G5" s="40" t="n">
-        <x:v>400</x:v>
-      </x:c>
-      <x:c r="H5" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="I5" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J5" s="40" t="n">
-        <x:v>0.18</x:v>
-      </x:c>
-      <x:c r="K5" s="37" t="str">
-        <x:v>Unlock: scatter_rig</x:v>
-      </x:c>
-      <x:c r="L5" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="37" t="str">
-        <x:v>Slug</x:v>
-      </x:c>
-      <x:c r="B6" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="C6" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="D6" s="40" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E6" s="40" t="n">
-        <x:v>2.20458553791887</x:v>
-      </x:c>
-      <x:c r="F6" s="40" t="n">
-        <x:v>648</x:v>
-      </x:c>
-      <x:c r="G6" s="40" t="n">
-        <x:v>620</x:v>
-      </x:c>
-      <x:c r="H6" s="40" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="I6" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J6" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K6" s="37" t="str">
-        <x:v>Unlock: slug_chamber</x:v>
-      </x:c>
-      <x:c r="L6" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="37" t="str">
-        <x:v>Incinerator</x:v>
-      </x:c>
-      <x:c r="B7" s="37" t="str">
-        <x:v>cone</x:v>
-      </x:c>
-      <x:c r="C7" s="37" t="str">
-        <x:v>cone, tick_damage</x:v>
-      </x:c>
-      <x:c r="D7" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E7" s="40" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="F7" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G7" s="40" t="n">
-        <x:v>220</x:v>
-      </x:c>
-      <x:c r="H7" s="40" t="n">
-        <x:v>0.72</x:v>
-      </x:c>
-      <x:c r="I7" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J7" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" s="37" t="str">
-        <x:v>Unlock ID: incinerator_core (missing in unlocks.json)</x:v>
-      </x:c>
-      <x:c r="L7" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="37" t="str">
-        <x:v>Beam Lance</x:v>
-      </x:c>
-      <x:c r="B8" s="37" t="str">
-        <x:v>beam</x:v>
-      </x:c>
-      <x:c r="C8" s="37" t="str">
-        <x:v>beam, tick_damage</x:v>
-      </x:c>
-      <x:c r="D8" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="40" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F8" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G8" s="40" t="n">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="H8" s="40" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="I8" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J8" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K8" s="37" t="str">
-        <x:v>Unlock ID: beam_lance (missing in unlocks.json)</x:v>
-      </x:c>
-      <x:c r="L8" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="37" t="str">
-        <x:v>Arc Caster</x:v>
-      </x:c>
-      <x:c r="B9" s="37" t="str">
-        <x:v>chain</x:v>
-      </x:c>
-      <x:c r="C9" s="37" t="str">
-        <x:v>chain</x:v>
-      </x:c>
-      <x:c r="D9" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E9" s="40" t="n">
-        <x:v>2.8</x:v>
-      </x:c>
-      <x:c r="F9" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G9" s="40" t="n">
-        <x:v>280</x:v>
-      </x:c>
-      <x:c r="H9" s="40" t="n">
-        <x:v>150</x:v>
-      </x:c>
-      <x:c r="I9" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J9" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K9" s="37" t="str">
-        <x:v>Unlock ID: arc_caster (missing in unlocks.json)</x:v>
-      </x:c>
-      <x:c r="L9" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:L1"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8082655e01be47e2"/>
-  </x:tableParts>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="26" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="10" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="10" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="42" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="80" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="str">
+        <v>Primary Weapons — Base Stats</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="36" t="str">
+        <v>Weapon</v>
+      </c>
+      <c r="B3" s="36" t="str">
+        <v>Behavior</v>
+      </c>
+      <c r="C3" s="36" t="str">
+        <v>Tags</v>
+      </c>
+      <c r="D3" s="36" t="str">
+        <v>Base Dmg</v>
+      </c>
+      <c r="E3" s="36" t="str">
+        <v>Base FR</v>
+      </c>
+      <c r="F3" s="36" t="str">
+        <v>Projectile Spd</v>
+      </c>
+      <c r="G3" s="36" t="str">
+        <v>Range</v>
+      </c>
+      <c r="H3" s="36" t="str">
+        <v>Area</v>
+      </c>
+      <c r="I3" s="36" t="str">
+        <v>Amount</v>
+      </c>
+      <c r="J3" s="36" t="str">
+        <v>Spread</v>
+      </c>
+      <c r="K3" s="36" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="L3" s="36" t="str">
+        <v>Source URL</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="str">
+        <v>Rifle</v>
+      </c>
+      <c r="B4" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="C4" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="D4" s="40">
+        <v>10</v>
+      </c>
+      <c r="E4" s="40" t="n">
+        <v>4.62962962962963</v>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>540</v>
+      </c>
+      <c r="G4" s="40" t="n">
+        <v>520</v>
+      </c>
+      <c r="H4" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="37" t="str"/>
+      <c r="L4" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="str">
+        <v>Scatter</v>
+      </c>
+      <c r="B5" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="C5" s="37" t="str">
+        <v>projectile, spread</v>
+      </c>
+      <c r="D5" s="40">
+        <v>10</v>
+      </c>
+      <c r="E5" s="40" t="n">
+        <v>3.42935528120713</v>
+      </c>
+      <c r="F5" s="40" t="n">
+        <v>513</v>
+      </c>
+      <c r="G5" s="40" t="n">
+        <v>400</v>
+      </c>
+      <c r="H5" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="40" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K5" s="37" t="str">
+        <v>Unlock: scatter_rig</v>
+      </c>
+      <c r="L5" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="str">
+        <v>Slug</v>
+      </c>
+      <c r="B6" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="C6" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="D6" s="40">
+        <v>20</v>
+      </c>
+      <c r="E6" s="40" t="n">
+        <v>2.20458553791887</v>
+      </c>
+      <c r="F6" s="40" t="n">
+        <v>648</v>
+      </c>
+      <c r="G6" s="40" t="n">
+        <v>620</v>
+      </c>
+      <c r="H6" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="37" t="str">
+        <v>Unlock: slug_chamber</v>
+      </c>
+      <c r="L6" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="str">
+        <v>Incinerator</v>
+      </c>
+      <c r="B7" s="37" t="str">
+        <v>cone</v>
+      </c>
+      <c r="C7" s="37" t="str">
+        <v>cone, tick_damage</v>
+      </c>
+      <c r="D7" s="40">
+        <v>10</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>220</v>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="37" t="str">
+        <v>Unlock ID: incinerator_core (missing in unlocks.json)</v>
+      </c>
+      <c r="L7" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="str">
+        <v>Beam Lance</v>
+      </c>
+      <c r="B8" s="37" t="str">
+        <v>beam</v>
+      </c>
+      <c r="C8" s="37" t="str">
+        <v>beam, tick_damage</v>
+      </c>
+      <c r="D8" s="40">
+        <v>10</v>
+      </c>
+      <c r="E8" s="40" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="40" t="n">
+        <v>460</v>
+      </c>
+      <c r="H8" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="I8" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="37" t="str">
+        <v>Unlock ID: beam_lance (missing in unlocks.json)</v>
+      </c>
+      <c r="L8" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="str">
+        <v>Arc Caster</v>
+      </c>
+      <c r="B9" s="37" t="str">
+        <v>chain</v>
+      </c>
+      <c r="C9" s="37" t="str">
+        <v>chain</v>
+      </c>
+      <c r="D9" s="40">
+        <v>10</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="40" t="n">
+        <v>280</v>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>150</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="37" t="str">
+        <v>Unlock ID: arc_caster (missing in unlocks.json)</v>
+      </c>
+      <c r="L9" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart ns1:id="R8082655e01be47e2"/>
+  </tableParts>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1421,321 +1421,326 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="34" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="80" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Secondary Weapons — Base Stats</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="36" t="str">
-        <x:v>Weapon</x:v>
-      </x:c>
-      <x:c r="B3" s="36" t="str">
-        <x:v>Family</x:v>
-      </x:c>
-      <x:c r="C3" s="36" t="str">
-        <x:v>Kind</x:v>
-      </x:c>
-      <x:c r="D3" s="36" t="str">
-        <x:v>Cooldown Mult</x:v>
-      </x:c>
-      <x:c r="E3" s="36" t="str">
-        <x:v>Projectile Speed</x:v>
-      </x:c>
-      <x:c r="F3" s="36" t="str">
-        <x:v>Damage Mult</x:v>
-      </x:c>
-      <x:c r="G3" s="36" t="str">
-        <x:v>Explosion Radius Mult</x:v>
-      </x:c>
-      <x:c r="H3" s="36" t="str">
-        <x:v>Fuse Time</x:v>
-      </x:c>
-      <x:c r="I3" s="36" t="str">
-        <x:v>Pulse Count</x:v>
-      </x:c>
-      <x:c r="J3" s="36" t="str">
-        <x:v>Cluster Blasts</x:v>
-      </x:c>
-      <x:c r="K3" s="36" t="str">
-        <x:v>Proximity Radius</x:v>
-      </x:c>
-      <x:c r="L3" s="36" t="str">
-        <x:v>Notes</x:v>
-      </x:c>
-      <x:c r="M3" s="36" t="str">
-        <x:v>Source URL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="37" t="str">
-        <x:v>Grenade</x:v>
-      </x:c>
-      <x:c r="B4" s="37" t="str">
-        <x:v>thrown</x:v>
-      </x:c>
-      <x:c r="C4" s="37" t="str">
-        <x:v>grenade</x:v>
-      </x:c>
-      <x:c r="D4" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E4" s="40" t="n">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F4" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G4" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H4" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I4" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J4" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K4" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L4" s="37" t="str"/>
-      <x:c r="M4" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="37" t="str">
-        <x:v>Cluster Grenade</x:v>
-      </x:c>
-      <x:c r="B5" s="37" t="str">
-        <x:v>thrown</x:v>
-      </x:c>
-      <x:c r="C5" s="37" t="str">
-        <x:v>cluster_grenade</x:v>
-      </x:c>
-      <x:c r="D5" s="40" t="n">
-        <x:v>0.92</x:v>
-      </x:c>
-      <x:c r="E5" s="40" t="n">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F5" s="40" t="n">
-        <x:v>0.8</x:v>
-      </x:c>
-      <x:c r="G5" s="40" t="n">
-        <x:v>0.78</x:v>
-      </x:c>
-      <x:c r="H5" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I5" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J5" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="K5" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L5" s="37" t="str">
-        <x:v>Unlock: cluster_grenades</x:v>
-      </x:c>
-      <x:c r="M5" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="37" t="str">
-        <x:v>Siege Grenade</x:v>
-      </x:c>
-      <x:c r="B6" s="37" t="str">
-        <x:v>thrown</x:v>
-      </x:c>
-      <x:c r="C6" s="37" t="str">
-        <x:v>siege_grenade</x:v>
-      </x:c>
-      <x:c r="D6" s="40" t="n">
-        <x:v>1.35</x:v>
-      </x:c>
-      <x:c r="E6" s="40" t="n">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="F6" s="40" t="n">
-        <x:v>1.1</x:v>
-      </x:c>
-      <x:c r="G6" s="40" t="n">
-        <x:v>1.35</x:v>
-      </x:c>
-      <x:c r="H6" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I6" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J6" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K6" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L6" s="37" t="str">
-        <x:v>Unlock: siege_grenades</x:v>
-      </x:c>
-      <x:c r="M6" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="37" t="str">
-        <x:v>Mine</x:v>
-      </x:c>
-      <x:c r="B7" s="37" t="str">
-        <x:v>proximity</x:v>
-      </x:c>
-      <x:c r="C7" s="37" t="str">
-        <x:v>mine</x:v>
-      </x:c>
-      <x:c r="D7" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E7" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F7" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G7" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H7" s="40" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="I7" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J7" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K7" s="40" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="L7" s="37" t="str"/>
-      <x:c r="M7" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="37" t="str">
-        <x:v>Shrapnel Mine</x:v>
-      </x:c>
-      <x:c r="B8" s="37" t="str">
-        <x:v>proximity</x:v>
-      </x:c>
-      <x:c r="C8" s="37" t="str">
-        <x:v>shrapnel_mine</x:v>
-      </x:c>
-      <x:c r="D8" s="40" t="n">
-        <x:v>0.92</x:v>
-      </x:c>
-      <x:c r="E8" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F8" s="40" t="n">
-        <x:v>0.82</x:v>
-      </x:c>
-      <x:c r="G8" s="40" t="n">
-        <x:v>0.82</x:v>
-      </x:c>
-      <x:c r="H8" s="40" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="I8" s="40" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J8" s="40" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="K8" s="40" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="L8" s="37" t="str">
-        <x:v>Unlock: cluster_shells</x:v>
-      </x:c>
-      <x:c r="M8" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="37" t="str">
-        <x:v>Heavy Mine</x:v>
-      </x:c>
-      <x:c r="B9" s="37" t="str">
-        <x:v>proximity</x:v>
-      </x:c>
-      <x:c r="C9" s="37" t="str">
-        <x:v>heavy_mine</x:v>
-      </x:c>
-      <x:c r="D9" s="40" t="n">
-        <x:v>1.3</x:v>
-      </x:c>
-      <x:c r="E9" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F9" s="40" t="n">
-        <x:v>1.15</x:v>
-      </x:c>
-      <x:c r="G9" s="40" t="n">
-        <x:v>1.35</x:v>
-      </x:c>
-      <x:c r="H9" s="40" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="I9" s="40" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="J9" s="40" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K9" s="40" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="L9" s="37" t="str">
-        <x:v>Unlock: siege_canister</x:v>
-      </x:c>
-      <x:c r="M9" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:L1"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fb9f0c0a74b4df1"/>
-  </x:tableParts>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="13" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="16" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="34" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="80" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="str">
+        <v>Secondary Weapons — Base Stats</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Shared secondary base damage is 30 before weapon damage_mult and passive flat bonuses.</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="36" t="str">
+        <v>Weapon</v>
+      </c>
+      <c r="B3" s="36" t="str">
+        <v>Family</v>
+      </c>
+      <c r="C3" s="36" t="str">
+        <v>Kind</v>
+      </c>
+      <c r="D3" s="36" t="str">
+        <v>Cooldown Mult</v>
+      </c>
+      <c r="E3" s="36" t="str">
+        <v>Projectile Speed</v>
+      </c>
+      <c r="F3" s="36" t="str">
+        <v>Damage Mult</v>
+      </c>
+      <c r="G3" s="36" t="str">
+        <v>Explosion Radius Mult</v>
+      </c>
+      <c r="H3" s="36" t="str">
+        <v>Fuse Time</v>
+      </c>
+      <c r="I3" s="36" t="str">
+        <v>Pulse Count</v>
+      </c>
+      <c r="J3" s="36" t="str">
+        <v>Cluster Blasts</v>
+      </c>
+      <c r="K3" s="36" t="str">
+        <v>Proximity Radius</v>
+      </c>
+      <c r="L3" s="36" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="M3" s="36" t="str">
+        <v>Source URL</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="str">
+        <v>Grenade</v>
+      </c>
+      <c r="B4" s="37" t="str">
+        <v>thrown</v>
+      </c>
+      <c r="C4" s="37" t="str">
+        <v>grenade</v>
+      </c>
+      <c r="D4" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="40" t="n">
+        <v>125</v>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="37" t="str"/>
+      <c r="M4" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="str">
+        <v>Cluster Grenade</v>
+      </c>
+      <c r="B5" s="37" t="str">
+        <v>thrown</v>
+      </c>
+      <c r="C5" s="37" t="str">
+        <v>cluster_grenade</v>
+      </c>
+      <c r="D5" s="40" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E5" s="40" t="n">
+        <v>125</v>
+      </c>
+      <c r="F5" s="40" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G5" s="40" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="H5" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="37" t="str">
+        <v>Unlock: cluster_grenades</v>
+      </c>
+      <c r="M5" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="str">
+        <v>Siege Grenade</v>
+      </c>
+      <c r="B6" s="37" t="str">
+        <v>thrown</v>
+      </c>
+      <c r="C6" s="37" t="str">
+        <v>siege_grenade</v>
+      </c>
+      <c r="D6" s="40" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="E6" s="40" t="n">
+        <v>125</v>
+      </c>
+      <c r="F6" s="40" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G6" s="40" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H6" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="37" t="str">
+        <v>Unlock: siege_grenades</v>
+      </c>
+      <c r="M6" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="str">
+        <v>Mine</v>
+      </c>
+      <c r="B7" s="37" t="str">
+        <v>proximity</v>
+      </c>
+      <c r="C7" s="37" t="str">
+        <v>mine</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="I7" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="40" t="n">
+        <v>52</v>
+      </c>
+      <c r="L7" s="37" t="str"/>
+      <c r="M7" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="str">
+        <v>Shrapnel Mine</v>
+      </c>
+      <c r="B8" s="37" t="str">
+        <v>proximity</v>
+      </c>
+      <c r="C8" s="37" t="str">
+        <v>shrapnel_mine</v>
+      </c>
+      <c r="D8" s="40" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E8" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="40" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G8" s="40" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="H8" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="I8" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="40" t="n">
+        <v>52</v>
+      </c>
+      <c r="L8" s="37" t="str">
+        <v>Unlock: cluster_shells</v>
+      </c>
+      <c r="M8" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="str">
+        <v>Heavy Mine</v>
+      </c>
+      <c r="B9" s="37" t="str">
+        <v>proximity</v>
+      </c>
+      <c r="C9" s="37" t="str">
+        <v>heavy_mine</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="G9" s="40" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="H9" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="I9" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="40" t="n">
+        <v>52</v>
+      </c>
+      <c r="L9" s="37" t="str">
+        <v>Unlock: siege_canister</v>
+      </c>
+      <c r="M9" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/weapons.json</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart ns1:id="R4fb9f0c0a74b4df1"/>
+  </tableParts>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2143,417 +2148,417 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="72" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="80" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="5" t="str">
-        <x:v>Implemented Passive Items</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="12" t="str">
-        <x:v>Passives are currently fixed effects, not levelled. All listed passives are non-stackable in data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="24" customHeight="1">
-      <x:c r="A3" s="36" t="str">
-        <x:v>Passive</x:v>
-      </x:c>
-      <x:c r="B3" s="36" t="str">
-        <x:v>Requirement / Tag Filter</x:v>
-      </x:c>
-      <x:c r="C3" s="36" t="str">
-        <x:v>Effect Domain</x:v>
-      </x:c>
-      <x:c r="D3" s="36" t="str">
-        <x:v>Stats / Trigger Behavior</x:v>
-      </x:c>
-      <x:c r="E3" s="36" t="str">
-        <x:v>Stackable</x:v>
-      </x:c>
-      <x:c r="F3" s="36" t="str">
-        <x:v>Source URL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="37" t="str">
-        <x:v>Overclocked Receiver</x:v>
-      </x:c>
-      <x:c r="B4" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C4" s="37" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-      <x:c r="D4" s="37" t="str">
-        <x:v>Primary FR x1.136</x:v>
-      </x:c>
-      <x:c r="E4" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F4" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="37" t="str">
-        <x:v>Rapid Loader</x:v>
-      </x:c>
-      <x:c r="B5" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C5" s="37" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-      <x:c r="D5" s="37" t="str">
-        <x:v>Primary FR x1.220</x:v>
-      </x:c>
-      <x:c r="E5" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F5" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="37" t="str">
-        <x:v>Tungsten Cores</x:v>
-      </x:c>
-      <x:c r="B6" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C6" s="37" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-      <x:c r="D6" s="37" t="str">
-        <x:v>Primary Dmg +2</x:v>
-      </x:c>
-      <x:c r="E6" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F6" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="37" t="str">
-        <x:v>Velocity Rig</x:v>
-      </x:c>
-      <x:c r="B7" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="C7" s="37" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-      <x:c r="D7" s="37" t="str">
-        <x:v>Projectile Spd x1.35; Primary FR x0.870</x:v>
-      </x:c>
-      <x:c r="E7" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F7" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="37" t="str">
-        <x:v>Blast Amplifier</x:v>
-      </x:c>
-      <x:c r="B8" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C8" s="37" t="str">
-        <x:v>passive_effects</x:v>
-      </x:c>
-      <x:c r="D8" s="37" t="str">
-        <x:v>Secondary explosion radius x1.3</x:v>
-      </x:c>
-      <x:c r="E8" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F8" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="37" t="str">
-        <x:v>Charged Payload</x:v>
-      </x:c>
-      <x:c r="B9" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C9" s="37" t="str">
-        <x:v>passive_effects</x:v>
-      </x:c>
-      <x:c r="D9" s="37" t="str">
-        <x:v>Secondary detonation Dmg +2</x:v>
-      </x:c>
-      <x:c r="E9" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F9" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="37" t="str">
-        <x:v>Quick Deploy</x:v>
-      </x:c>
-      <x:c r="B10" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C10" s="37" t="str">
-        <x:v>passive_effects</x:v>
-      </x:c>
-      <x:c r="D10" s="37" t="str">
-        <x:v>Secondary CD x0.7</x:v>
-      </x:c>
-      <x:c r="E10" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F10" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="37" t="str">
-        <x:v>Quick Release Valve</x:v>
-      </x:c>
-      <x:c r="B11" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C11" s="37" t="str">
-        <x:v>passive_effects</x:v>
-      </x:c>
-      <x:c r="D11" s="37" t="str">
-        <x:v>Secondary CD x0.8</x:v>
-      </x:c>
-      <x:c r="E11" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F11" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="37" t="str">
-        <x:v>Chain Reaction</x:v>
-      </x:c>
-      <x:c r="B12" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C12" s="37" t="str">
-        <x:v>mixed</x:v>
-      </x:c>
-      <x:c r="D12" s="37" t="str">
-        <x:v>Primary Dmg +1; Secondary explosion radius x1.2</x:v>
-      </x:c>
-      <x:c r="E12" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F12" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="37" t="str">
-        <x:v>High Velocity Rounds</x:v>
-      </x:c>
-      <x:c r="B13" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="C13" s="37" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-      <x:c r="D13" s="37" t="str">
-        <x:v>Projectile Spd x1.2; Primary Dmg +1</x:v>
-      </x:c>
-      <x:c r="E13" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F13" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="37" t="str">
-        <x:v>Armor Piercing Rounds</x:v>
-      </x:c>
-      <x:c r="B14" s="37" t="str">
-        <x:v>projectile</x:v>
-      </x:c>
-      <x:c r="C14" s="37" t="str">
-        <x:v>effects</x:v>
-      </x:c>
-      <x:c r="D14" s="37" t="str">
-        <x:v>Pierce count +1</x:v>
-      </x:c>
-      <x:c r="E14" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F14" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="37" t="str">
-        <x:v>Ember Bloom</x:v>
-      </x:c>
-      <x:c r="B15" s="37" t="str">
-        <x:v>cone</x:v>
-      </x:c>
-      <x:c r="C15" s="37" t="str">
-        <x:v>trigger on_fire</x:v>
-      </x:c>
-      <x:c r="D15" s="37" t="str">
-        <x:v>Every 3rd fire: bonus cone; Dmg 1; Rng 150; Area 0.52; Amt 1</x:v>
-      </x:c>
-      <x:c r="E15" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F15" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="37" t="str">
-        <x:v>Feedback Arc</x:v>
-      </x:c>
-      <x:c r="B16" s="37" t="str">
-        <x:v>beam</x:v>
-      </x:c>
-      <x:c r="C16" s="37" t="str">
-        <x:v>trigger on_hit</x:v>
-      </x:c>
-      <x:c r="D16" s="37" t="str">
-        <x:v>Every 2 hits; 50% chance; 0.2s CD: bonus chain; Dmg 1; Rng 170; Area 120; Amt 2</x:v>
-      </x:c>
-      <x:c r="E16" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F16" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="37" t="str">
-        <x:v>Culling Burst</x:v>
-      </x:c>
-      <x:c r="B17" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C17" s="37" t="str">
-        <x:v>trigger on_kill</x:v>
-      </x:c>
-      <x:c r="D17" s="37" t="str">
-        <x:v>On kill; 0.2s CD: explosion; Dmg 1; Radius 58; max targets 3</x:v>
-      </x:c>
-      <x:c r="E17" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F17" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="37" t="str">
-        <x:v>Detonation Web</x:v>
-      </x:c>
-      <x:c r="B18" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C18" s="37" t="str">
-        <x:v>trigger on_explosion</x:v>
-      </x:c>
-      <x:c r="D18" s="37" t="str">
-        <x:v>On explosion; 0.25s CD: bonus chain; Dmg 1; Rng 150; Area 110; Amt 2</x:v>
-      </x:c>
-      <x:c r="E18" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F18" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="37" t="str">
-        <x:v>Ablative Coating</x:v>
-      </x:c>
-      <x:c r="B19" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C19" s="37" t="str">
-        <x:v>passive_effects</x:v>
-      </x:c>
-      <x:c r="D19" s="37" t="str">
-        <x:v>Max HP +2; immediate restore by that amount</x:v>
-      </x:c>
-      <x:c r="E19" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F19" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="37" t="str">
-        <x:v>Reinforced Plating</x:v>
-      </x:c>
-      <x:c r="B20" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C20" s="37" t="str">
-        <x:v>passive_effects</x:v>
-      </x:c>
-      <x:c r="D20" s="37" t="str">
-        <x:v>Max HP +1; immediate heal by that amount</x:v>
-      </x:c>
-      <x:c r="E20" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F20" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="37" t="str">
-        <x:v>Sprint Servos</x:v>
-      </x:c>
-      <x:c r="B21" s="37" t="str">
-        <x:v>none</x:v>
-      </x:c>
-      <x:c r="C21" s="37" t="str">
-        <x:v>passive_effects</x:v>
-      </x:c>
-      <x:c r="D21" s="37" t="str">
-        <x:v>Move speed x1.18</x:v>
-      </x:c>
-      <x:c r="E21" s="37" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="F21" s="37" t="str">
-        <x:v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</x:v>
-      </x:c>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:L1"/>
-    <x:mergeCell ref="A2:L2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66fab57bec5f4ccc"/>
-  </x:tableParts>
-</x:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="72" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="80" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="5" t="str">
+        <v>Implemented Passive Items</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="12" t="str">
+        <v>Passives are currently fixed effects, not levelled. All listed passives are non-stackable in data.</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="36" t="str">
+        <v>Passive</v>
+      </c>
+      <c r="B3" s="36" t="str">
+        <v>Requirement / Tag Filter</v>
+      </c>
+      <c r="C3" s="36" t="str">
+        <v>Effect Domain</v>
+      </c>
+      <c r="D3" s="36" t="str">
+        <v>Stats / Trigger Behavior</v>
+      </c>
+      <c r="E3" s="36" t="str">
+        <v>Stackable</v>
+      </c>
+      <c r="F3" s="36" t="str">
+        <v>Source URL</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="str">
+        <v>Overclocked Receiver</v>
+      </c>
+      <c r="B4" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C4" s="37" t="str">
+        <v>effects</v>
+      </c>
+      <c r="D4" s="37" t="str">
+        <v>Primary FR x1.136</v>
+      </c>
+      <c r="E4" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F4" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="str">
+        <v>Rapid Loader</v>
+      </c>
+      <c r="B5" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C5" s="37" t="str">
+        <v>effects</v>
+      </c>
+      <c r="D5" s="37" t="str">
+        <v>Primary FR x1.220</v>
+      </c>
+      <c r="E5" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F5" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="str">
+        <v>Tungsten Cores</v>
+      </c>
+      <c r="B6" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C6" s="37" t="str">
+        <v>effects</v>
+      </c>
+      <c r="D6" s="37" t="str">
+        <v>Primary Dmg +20</v>
+      </c>
+      <c r="E6" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F6" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="str">
+        <v>Velocity Rig</v>
+      </c>
+      <c r="B7" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="C7" s="37" t="str">
+        <v>effects</v>
+      </c>
+      <c r="D7" s="37" t="str">
+        <v>Projectile Spd x1.35; Primary FR x0.870</v>
+      </c>
+      <c r="E7" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F7" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="str">
+        <v>Blast Amplifier</v>
+      </c>
+      <c r="B8" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C8" s="37" t="str">
+        <v>passive_effects</v>
+      </c>
+      <c r="D8" s="37" t="str">
+        <v>Secondary explosion radius x1.3</v>
+      </c>
+      <c r="E8" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F8" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="str">
+        <v>Charged Payload</v>
+      </c>
+      <c r="B9" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C9" s="37" t="str">
+        <v>passive_effects</v>
+      </c>
+      <c r="D9" s="37" t="str">
+        <v>Secondary detonation Dmg +20</v>
+      </c>
+      <c r="E9" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F9" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="str">
+        <v>Quick Deploy</v>
+      </c>
+      <c r="B10" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C10" s="37" t="str">
+        <v>passive_effects</v>
+      </c>
+      <c r="D10" s="37" t="str">
+        <v>Secondary CD x0.7</v>
+      </c>
+      <c r="E10" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F10" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="str">
+        <v>Quick Release Valve</v>
+      </c>
+      <c r="B11" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C11" s="37" t="str">
+        <v>passive_effects</v>
+      </c>
+      <c r="D11" s="37" t="str">
+        <v>Secondary CD x0.8</v>
+      </c>
+      <c r="E11" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F11" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="37" t="str">
+        <v>Chain Reaction</v>
+      </c>
+      <c r="B12" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C12" s="37" t="str">
+        <v>mixed</v>
+      </c>
+      <c r="D12" s="37" t="str">
+        <v>Primary Dmg +10; Secondary explosion radius x1.2</v>
+      </c>
+      <c r="E12" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F12" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="str">
+        <v>High Velocity Rounds</v>
+      </c>
+      <c r="B13" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="C13" s="37" t="str">
+        <v>effects</v>
+      </c>
+      <c r="D13" s="37" t="str">
+        <v>Projectile Spd x1.2; Primary Dmg +10</v>
+      </c>
+      <c r="E13" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F13" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="37" t="str">
+        <v>Armor Piercing Rounds</v>
+      </c>
+      <c r="B14" s="37" t="str">
+        <v>projectile</v>
+      </c>
+      <c r="C14" s="37" t="str">
+        <v>effects</v>
+      </c>
+      <c r="D14" s="37" t="str">
+        <v>Pierce count +1</v>
+      </c>
+      <c r="E14" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F14" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="str">
+        <v>Ember Bloom</v>
+      </c>
+      <c r="B15" s="37" t="str">
+        <v>cone</v>
+      </c>
+      <c r="C15" s="37" t="str">
+        <v>trigger on_fire</v>
+      </c>
+      <c r="D15" s="37" t="str">
+        <v>Every 3rd fire: bonus cone; Dmg 10; Rng 150; Area 0.52; Amt 1</v>
+      </c>
+      <c r="E15" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F15" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="str">
+        <v>Feedback Arc</v>
+      </c>
+      <c r="B16" s="37" t="str">
+        <v>beam</v>
+      </c>
+      <c r="C16" s="37" t="str">
+        <v>trigger on_hit</v>
+      </c>
+      <c r="D16" s="37" t="str">
+        <v>Every 2 hits; 50% chance; 0.2s CD: bonus chain; Dmg 10; Rng 170; Area 120; Amt 2</v>
+      </c>
+      <c r="E16" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F16" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="str">
+        <v>Culling Burst</v>
+      </c>
+      <c r="B17" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C17" s="37" t="str">
+        <v>trigger on_kill</v>
+      </c>
+      <c r="D17" s="37" t="str">
+        <v>On kill; 0.2s CD: explosion; Dmg 10; Radius 58; max targets 3</v>
+      </c>
+      <c r="E17" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F17" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="37" t="str">
+        <v>Detonation Web</v>
+      </c>
+      <c r="B18" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C18" s="37" t="str">
+        <v>trigger on_explosion</v>
+      </c>
+      <c r="D18" s="37" t="str">
+        <v>On explosion; 0.25s CD: bonus chain; Dmg 10; Rng 150; Area 110; Amt 2</v>
+      </c>
+      <c r="E18" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F18" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="37" t="str">
+        <v>Ablative Coating</v>
+      </c>
+      <c r="B19" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C19" s="37" t="str">
+        <v>passive_effects</v>
+      </c>
+      <c r="D19" s="37" t="str">
+        <v>Max HP +20; immediate restore by that amount</v>
+      </c>
+      <c r="E19" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F19" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="37" t="str">
+        <v>Reinforced Plating</v>
+      </c>
+      <c r="B20" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C20" s="37" t="str">
+        <v>passive_effects</v>
+      </c>
+      <c r="D20" s="37" t="str">
+        <v>Max HP +10; immediate heal by that amount</v>
+      </c>
+      <c r="E20" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F20" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="37" t="str">
+        <v>Sprint Servos</v>
+      </c>
+      <c r="B21" s="37" t="str">
+        <v>none</v>
+      </c>
+      <c r="C21" s="37" t="str">
+        <v>passive_effects</v>
+      </c>
+      <c r="D21" s="37" t="str">
+        <v>Move speed x1.18</v>
+      </c>
+      <c r="E21" s="37" t="str">
+        <v>No</v>
+      </c>
+      <c r="F21" s="37" t="str">
+        <v>https://github.com/snaxico/project-twin-stick/blob/codex/primary-ruleset-plan/data/passives.json</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart ns1:id="R66fab57bec5f4ccc"/>
+  </tableParts>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>